<commit_message>
update: 2026/07/08 周三 20:35:27.60
</commit_message>
<xml_diff>
--- a/source/9、人数基数/人数基数-4月.xlsx
+++ b/source/9、人数基数/人数基数-4月.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="21550" windowHeight="10200"/>
+    <workbookView windowWidth="22400" windowHeight="10200"/>
   </bookViews>
   <sheets>
     <sheet name="人数基数模板" sheetId="1" r:id="rId1"/>
@@ -1326,10 +1326,10 @@
         <v>7</v>
       </c>
       <c r="D2" s="2">
-        <v>863</v>
+        <v>901</v>
       </c>
       <c r="E2" s="1">
-        <v>863</v>
+        <v>901</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1343,10 +1343,10 @@
         <v>7</v>
       </c>
       <c r="D3" s="2">
-        <v>751</v>
+        <v>711</v>
       </c>
       <c r="E3" s="1">
-        <v>751</v>
+        <v>711</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1360,10 +1360,10 @@
         <v>7</v>
       </c>
       <c r="D4" s="2">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="E4" s="1">
-        <v>570</v>
+        <v>573</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1377,10 +1377,10 @@
         <v>7</v>
       </c>
       <c r="D5" s="2">
-        <v>632</v>
+        <v>668</v>
       </c>
       <c r="E5" s="1">
-        <v>632</v>
+        <v>668</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1394,10 +1394,10 @@
         <v>7</v>
       </c>
       <c r="D6" s="2">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="E6" s="1">
-        <v>440</v>
+        <v>437</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1411,10 +1411,10 @@
         <v>7</v>
       </c>
       <c r="D7" s="2">
-        <v>1804</v>
+        <v>1818</v>
       </c>
       <c r="E7" s="1">
-        <v>1804</v>
+        <v>1818</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1428,10 +1428,10 @@
         <v>7</v>
       </c>
       <c r="D8" s="2">
-        <v>1165</v>
+        <v>1202</v>
       </c>
       <c r="E8" s="1">
-        <v>1165</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1445,10 +1445,10 @@
         <v>7</v>
       </c>
       <c r="D9" s="2">
-        <v>2430</v>
+        <v>2462</v>
       </c>
       <c r="E9" s="1">
-        <v>2430</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1462,10 +1462,10 @@
         <v>7</v>
       </c>
       <c r="D10" s="2">
-        <v>935</v>
+        <v>937</v>
       </c>
       <c r="E10" s="1">
-        <v>935</v>
+        <v>937</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1479,10 +1479,10 @@
         <v>7</v>
       </c>
       <c r="D11" s="2">
-        <v>1128</v>
+        <v>1085</v>
       </c>
       <c r="E11" s="1">
-        <v>1128</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1496,10 +1496,10 @@
         <v>7</v>
       </c>
       <c r="D12" s="2">
-        <v>535</v>
+        <v>528</v>
       </c>
       <c r="E12" s="1">
-        <v>535</v>
+        <v>528</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1513,10 +1513,10 @@
         <v>7</v>
       </c>
       <c r="D13" s="2">
-        <v>797</v>
+        <v>819</v>
       </c>
       <c r="E13" s="1">
-        <v>797</v>
+        <v>819</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -1530,10 +1530,10 @@
         <v>7</v>
       </c>
       <c r="D14" s="2">
-        <v>909</v>
+        <v>894</v>
       </c>
       <c r="E14" s="1">
-        <v>909</v>
+        <v>894</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -1547,10 +1547,10 @@
         <v>7</v>
       </c>
       <c r="D15" s="2">
-        <v>586</v>
+        <v>571</v>
       </c>
       <c r="E15" s="1">
-        <v>586</v>
+        <v>571</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -1564,10 +1564,10 @@
         <v>7</v>
       </c>
       <c r="D16" s="2">
-        <v>1236</v>
+        <v>1219</v>
       </c>
       <c r="E16" s="1">
-        <v>1236</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1581,10 +1581,10 @@
         <v>7</v>
       </c>
       <c r="D17" s="2">
-        <v>856</v>
+        <v>895</v>
       </c>
       <c r="E17" s="1">
-        <v>856</v>
+        <v>895</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -1598,10 +1598,10 @@
         <v>7</v>
       </c>
       <c r="D18" s="2">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E18" s="1">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1615,10 +1615,10 @@
         <v>7</v>
       </c>
       <c r="D19" s="2">
-        <v>984</v>
+        <v>971</v>
       </c>
       <c r="E19" s="1">
-        <v>984</v>
+        <v>971</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -1632,10 +1632,10 @@
         <v>7</v>
       </c>
       <c r="D20" s="2">
-        <v>1204</v>
+        <v>1177</v>
       </c>
       <c r="E20" s="1">
-        <v>1204</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1649,10 +1649,10 @@
         <v>7</v>
       </c>
       <c r="D21" s="2">
-        <v>699</v>
+        <v>801</v>
       </c>
       <c r="E21" s="1">
-        <v>699</v>
+        <v>801</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1666,10 +1666,10 @@
         <v>7</v>
       </c>
       <c r="D22" s="2">
-        <v>1043</v>
+        <v>1031</v>
       </c>
       <c r="E22" s="1">
-        <v>1043</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1683,10 +1683,10 @@
         <v>7</v>
       </c>
       <c r="D23" s="2">
-        <v>388</v>
+        <v>364</v>
       </c>
       <c r="E23" s="1">
-        <v>388</v>
+        <v>364</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1700,10 +1700,10 @@
         <v>7</v>
       </c>
       <c r="D24" s="2">
-        <v>514</v>
+        <v>499</v>
       </c>
       <c r="E24" s="1">
-        <v>514</v>
+        <v>499</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1717,10 +1717,10 @@
         <v>7</v>
       </c>
       <c r="D25" s="2">
-        <v>1113</v>
+        <v>1086</v>
       </c>
       <c r="E25" s="1">
-        <v>1113</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1734,10 +1734,10 @@
         <v>7</v>
       </c>
       <c r="D26" s="2">
-        <v>993</v>
+        <v>949</v>
       </c>
       <c r="E26" s="1">
-        <v>993</v>
+        <v>949</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -1751,10 +1751,10 @@
         <v>7</v>
       </c>
       <c r="D27" s="2">
-        <v>952</v>
+        <v>980</v>
       </c>
       <c r="E27" s="1">
-        <v>952</v>
+        <v>980</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -1768,10 +1768,10 @@
         <v>7</v>
       </c>
       <c r="D28" s="2">
-        <v>378</v>
+        <v>345</v>
       </c>
       <c r="E28" s="1">
-        <v>378</v>
+        <v>345</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -1785,10 +1785,10 @@
         <v>7</v>
       </c>
       <c r="D29" s="2">
-        <v>662</v>
+        <v>672</v>
       </c>
       <c r="E29" s="1">
-        <v>662</v>
+        <v>672</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -1802,10 +1802,10 @@
         <v>7</v>
       </c>
       <c r="D30" s="2">
-        <v>429</v>
+        <v>409</v>
       </c>
       <c r="E30" s="1">
-        <v>429</v>
+        <v>409</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -1819,10 +1819,10 @@
         <v>7</v>
       </c>
       <c r="D31" s="2">
-        <v>1012</v>
+        <v>1085</v>
       </c>
       <c r="E31" s="1">
-        <v>1012</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -1836,10 +1836,10 @@
         <v>7</v>
       </c>
       <c r="D32" s="2">
-        <v>466</v>
+        <v>451</v>
       </c>
       <c r="E32" s="1">
-        <v>466</v>
+        <v>451</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -1853,10 +1853,10 @@
         <v>7</v>
       </c>
       <c r="D33" s="2">
-        <v>1033</v>
+        <v>1005</v>
       </c>
       <c r="E33" s="1">
-        <v>1033</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -1870,10 +1870,10 @@
         <v>7</v>
       </c>
       <c r="D34" s="2">
-        <v>438</v>
+        <v>428</v>
       </c>
       <c r="E34" s="1">
-        <v>438</v>
+        <v>428</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -1887,10 +1887,10 @@
         <v>7</v>
       </c>
       <c r="D35" s="2">
-        <v>933</v>
+        <v>897</v>
       </c>
       <c r="E35" s="1">
-        <v>933</v>
+        <v>897</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -1904,10 +1904,10 @@
         <v>7</v>
       </c>
       <c r="D36" s="2">
-        <v>2157</v>
+        <v>2135</v>
       </c>
       <c r="E36" s="1">
-        <v>2157</v>
+        <v>2135</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -1921,10 +1921,10 @@
         <v>7</v>
       </c>
       <c r="D37" s="2">
-        <v>424</v>
+        <v>416</v>
       </c>
       <c r="E37" s="1">
-        <v>424</v>
+        <v>416</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -1938,10 +1938,10 @@
         <v>7</v>
       </c>
       <c r="D38" s="2">
-        <v>1209</v>
+        <v>1182</v>
       </c>
       <c r="E38" s="1">
-        <v>1209</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -1955,10 +1955,10 @@
         <v>7</v>
       </c>
       <c r="D39" s="2">
-        <v>1652</v>
+        <v>1571</v>
       </c>
       <c r="E39" s="1">
-        <v>1652</v>
+        <v>1571</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -1972,10 +1972,10 @@
         <v>7</v>
       </c>
       <c r="D40" s="2">
-        <v>976</v>
+        <v>959</v>
       </c>
       <c r="E40" s="1">
-        <v>976</v>
+        <v>959</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -1989,10 +1989,10 @@
         <v>7</v>
       </c>
       <c r="D41" s="2">
-        <v>1181</v>
+        <v>1194</v>
       </c>
       <c r="E41" s="1">
-        <v>1181</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -2006,10 +2006,10 @@
         <v>7</v>
       </c>
       <c r="D42" s="2">
-        <v>420</v>
+        <v>390</v>
       </c>
       <c r="E42" s="1">
-        <v>420</v>
+        <v>390</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -2023,10 +2023,10 @@
         <v>7</v>
       </c>
       <c r="D43" s="2">
-        <v>350</v>
+        <v>335</v>
       </c>
       <c r="E43" s="1">
-        <v>350</v>
+        <v>335</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -2040,10 +2040,10 @@
         <v>7</v>
       </c>
       <c r="D44" s="2">
-        <v>1278</v>
+        <v>1216</v>
       </c>
       <c r="E44" s="1">
-        <v>1278</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -2057,10 +2057,10 @@
         <v>7</v>
       </c>
       <c r="D45" s="2">
-        <v>1531</v>
+        <v>1492</v>
       </c>
       <c r="E45" s="1">
-        <v>1531</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -2074,10 +2074,10 @@
         <v>7</v>
       </c>
       <c r="D46" s="2">
-        <v>527</v>
+        <v>560</v>
       </c>
       <c r="E46" s="1">
-        <v>527</v>
+        <v>560</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -2091,10 +2091,10 @@
         <v>7</v>
       </c>
       <c r="D47" s="2">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="E47" s="1">
-        <v>377</v>
+        <v>374</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -2108,10 +2108,10 @@
         <v>7</v>
       </c>
       <c r="D48" s="2">
-        <v>1125</v>
+        <v>1103</v>
       </c>
       <c r="E48" s="1">
-        <v>1125</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -2125,10 +2125,10 @@
         <v>7</v>
       </c>
       <c r="D49" s="2">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E49" s="1">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -2142,10 +2142,10 @@
         <v>7</v>
       </c>
       <c r="D50" s="2">
-        <v>492</v>
+        <v>509</v>
       </c>
       <c r="E50" s="1">
-        <v>492</v>
+        <v>509</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -2159,10 +2159,10 @@
         <v>7</v>
       </c>
       <c r="D51" s="2">
-        <v>578</v>
+        <v>603</v>
       </c>
       <c r="E51" s="1">
-        <v>578</v>
+        <v>603</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -2176,10 +2176,10 @@
         <v>7</v>
       </c>
       <c r="D52" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E52" s="1">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -2193,10 +2193,10 @@
         <v>7</v>
       </c>
       <c r="D53" s="2">
-        <v>335</v>
+        <v>322</v>
       </c>
       <c r="E53" s="1">
-        <v>335</v>
+        <v>322</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -2210,10 +2210,10 @@
         <v>7</v>
       </c>
       <c r="D54" s="2">
-        <v>844</v>
+        <v>820</v>
       </c>
       <c r="E54" s="1">
-        <v>844</v>
+        <v>820</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -2227,10 +2227,10 @@
         <v>7</v>
       </c>
       <c r="D55" s="2">
-        <v>356</v>
+        <v>345</v>
       </c>
       <c r="E55" s="1">
-        <v>356</v>
+        <v>345</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -2244,10 +2244,10 @@
         <v>7</v>
       </c>
       <c r="D56" s="2">
-        <v>544</v>
+        <v>532</v>
       </c>
       <c r="E56" s="1">
-        <v>544</v>
+        <v>532</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -2261,10 +2261,10 @@
         <v>7</v>
       </c>
       <c r="D57" s="2">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="E57" s="1">
-        <v>238</v>
+        <v>227</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -2278,10 +2278,10 @@
         <v>7</v>
       </c>
       <c r="D58" s="2">
-        <v>536</v>
+        <v>489</v>
       </c>
       <c r="E58" s="1">
-        <v>536</v>
+        <v>489</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -2295,10 +2295,10 @@
         <v>7</v>
       </c>
       <c r="D59" s="2">
-        <v>552</v>
+        <v>560</v>
       </c>
       <c r="E59" s="1">
-        <v>552</v>
+        <v>560</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -2312,10 +2312,10 @@
         <v>7</v>
       </c>
       <c r="D60" s="2">
-        <v>980</v>
+        <v>1019</v>
       </c>
       <c r="E60" s="1">
-        <v>980</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -2329,10 +2329,10 @@
         <v>67</v>
       </c>
       <c r="D61" s="2">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="E61" s="1">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -2346,10 +2346,10 @@
         <v>67</v>
       </c>
       <c r="D62" s="2">
-        <v>664</v>
+        <v>624</v>
       </c>
       <c r="E62" s="1">
-        <v>664</v>
+        <v>624</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -2363,10 +2363,10 @@
         <v>67</v>
       </c>
       <c r="D63" s="2">
-        <v>588</v>
+        <v>561</v>
       </c>
       <c r="E63" s="1">
-        <v>588</v>
+        <v>561</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -2380,10 +2380,10 @@
         <v>67</v>
       </c>
       <c r="D64" s="2">
-        <v>1339</v>
+        <v>1423</v>
       </c>
       <c r="E64" s="1">
-        <v>1339</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -2397,10 +2397,10 @@
         <v>67</v>
       </c>
       <c r="D65" s="2">
-        <v>371</v>
+        <v>416</v>
       </c>
       <c r="E65" s="1">
-        <v>371</v>
+        <v>416</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -2414,10 +2414,10 @@
         <v>67</v>
       </c>
       <c r="D66" s="2">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="E66" s="1">
-        <v>316</v>
+        <v>308</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -2431,10 +2431,10 @@
         <v>67</v>
       </c>
       <c r="D67" s="2">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="E67" s="1">
-        <v>559</v>
+        <v>563</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -2448,10 +2448,10 @@
         <v>67</v>
       </c>
       <c r="D68" s="2">
-        <v>308</v>
+        <v>294</v>
       </c>
       <c r="E68" s="1">
-        <v>308</v>
+        <v>294</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -2465,10 +2465,10 @@
         <v>67</v>
       </c>
       <c r="D69" s="2">
-        <v>1891</v>
+        <v>1804</v>
       </c>
       <c r="E69" s="1">
-        <v>1891</v>
+        <v>1804</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -2482,10 +2482,10 @@
         <v>67</v>
       </c>
       <c r="D70" s="2">
-        <v>305</v>
+        <v>294</v>
       </c>
       <c r="E70" s="1">
-        <v>305</v>
+        <v>294</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -2499,10 +2499,10 @@
         <v>67</v>
       </c>
       <c r="D71" s="2">
-        <v>275</v>
+        <v>291</v>
       </c>
       <c r="E71" s="1">
-        <v>275</v>
+        <v>291</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -2533,10 +2533,10 @@
         <v>67</v>
       </c>
       <c r="D73" s="2">
-        <v>572</v>
+        <v>559</v>
       </c>
       <c r="E73" s="1">
-        <v>572</v>
+        <v>559</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -2550,10 +2550,10 @@
         <v>67</v>
       </c>
       <c r="D74" s="2">
-        <v>391</v>
+        <v>356</v>
       </c>
       <c r="E74" s="1">
-        <v>391</v>
+        <v>356</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -2567,10 +2567,10 @@
         <v>67</v>
       </c>
       <c r="D75" s="2">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="E75" s="1">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -2584,10 +2584,10 @@
         <v>67</v>
       </c>
       <c r="D76" s="2">
-        <v>252</v>
+        <v>225</v>
       </c>
       <c r="E76" s="1">
-        <v>252</v>
+        <v>225</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -2601,10 +2601,10 @@
         <v>67</v>
       </c>
       <c r="D77" s="2">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="E77" s="1">
-        <v>290</v>
+        <v>287</v>
       </c>
     </row>
   </sheetData>

</xml_diff>